<commit_message>
Fix feature cross-references in the release backlog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRM7gnnA9AXrzoXHdE9dQs
</commit_message>
<xml_diff>
--- a/docs/business-analysis/backlog/backlog.xlsx
+++ b/docs/business-analysis/backlog/backlog.xlsx
@@ -1624,7 +1624,7 @@
 - Payment schedule as % of amount per milestone
 - Contract signing status
 - Project created with budget and project manager
-Not in this feature: Splitting one application into several projects → F30C
+Not in this feature: Splitting one application into several projects → F33
 Depends on: F16
 BRD use cases: UC67, UC69, UC70, UC71</t>
         </is>
@@ -1755,7 +1755,7 @@
 - Charity submits task progress, evidence files and milestone reports in the portal
 - Project manager verifies evidence: accept or return with note
 - Milestone approved → its payment becomes due
-Not in this feature: Indicators → F30C
+Not in this feature: Indicators → F33
 Depends on: F18
 BRD use cases: UC47, UC75, UC76</t>
         </is>

</xml_diff>